<commit_message>
added dim User Type
</commit_message>
<xml_diff>
--- a/docs/Citibike Data Map.xlsx
+++ b/docs/Citibike Data Map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/florentin/Desktop/Entwicklung/Repos/Citibike_Project/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7202B6B-DC83-7F4E-AF11-4135061B73F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F73CF8-41C7-EB48-A6F8-0D44980755E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="660" windowWidth="38640" windowHeight="17340" xr2:uid="{A950CCA5-45F8-463E-BCD8-1FA9D9B98C57}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17340" xr2:uid="{A950CCA5-45F8-463E-BCD8-1FA9D9B98C57}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="77">
   <si>
     <t>Target</t>
   </si>
@@ -261,6 +261,12 @@
   </si>
   <si>
     <t>CASE WHEN precipitation_mm = 0 THEN '1_Trocken' WHEN precipitation_mm &gt; 0 AND precipitation_mm &lt;= 5 THEN '2_Leichter Regen (0-5mm)' ELSE '3_Starker Regen (&gt;5mm)' END</t>
+  </si>
+  <si>
+    <t>dim_user_type</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT member_casual AS user_type - Natural Key</t>
   </si>
 </sst>
 </file>
@@ -313,7 +319,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -538,59 +544,31 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
       <right style="medium">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -619,7 +597,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -651,9 +629,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -672,25 +660,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1028,7 +1000,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -1043,20 +1015,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="15" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="16" t="s">
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="20" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1088,7 +1060,7 @@
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="17"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
@@ -1118,7 +1090,7 @@
       <c r="I3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1150,7 +1122,7 @@
       <c r="I4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="20" t="s">
+      <c r="J4" s="13" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1182,7 +1154,7 @@
       <c r="I5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="13" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1214,7 +1186,7 @@
       <c r="I6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="20" t="s">
+      <c r="J6" s="13" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1246,7 +1218,7 @@
       <c r="I7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="20" t="s">
+      <c r="J7" s="13" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1278,7 +1250,7 @@
       <c r="I8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="20" t="s">
+      <c r="J8" s="13" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1310,7 +1282,7 @@
       <c r="I9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="20" t="s">
+      <c r="J9" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1327,7 +1299,7 @@
       <c r="D10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="1">
         <v>1</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -1342,7 +1314,7 @@
       <c r="I10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J10" s="20" t="s">
+      <c r="J10" s="13" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1359,7 +1331,7 @@
       <c r="D11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="1">
         <v>1</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -1368,13 +1340,13 @@
       <c r="G11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="11" t="s">
         <v>41</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J11" s="20" t="s">
+      <c r="J11" s="13" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1391,7 +1363,7 @@
       <c r="D12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="1">
         <v>1</v>
       </c>
       <c r="F12" s="2" t="s">
@@ -1406,7 +1378,7 @@
       <c r="I12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="20" t="s">
+      <c r="J12" s="13" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1423,7 +1395,7 @@
       <c r="D13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="1">
         <v>1</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -1438,7 +1410,7 @@
       <c r="I13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J13" s="20" t="s">
+      <c r="J13" s="13" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1455,7 +1427,7 @@
       <c r="D14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="1">
         <v>1</v>
       </c>
       <c r="F14" s="2" t="s">
@@ -1470,7 +1442,7 @@
       <c r="I14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J14" s="20" t="s">
+      <c r="J14" s="13" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1487,7 +1459,7 @@
       <c r="D15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="1">
         <v>1</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -1502,7 +1474,7 @@
       <c r="I15" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J15" s="20" t="s">
+      <c r="J15" s="13" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1519,7 +1491,7 @@
       <c r="D16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="1">
         <v>1</v>
       </c>
       <c r="F16" s="2" t="s">
@@ -1534,7 +1506,7 @@
       <c r="I16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J16" s="20" t="s">
+      <c r="J16" s="13" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1551,7 +1523,7 @@
       <c r="D17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="1">
         <v>1</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -1566,7 +1538,7 @@
       <c r="I17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J17" s="20" t="s">
+      <c r="J17" s="13" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1583,7 +1555,7 @@
       <c r="D18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="1">
         <v>1</v>
       </c>
       <c r="F18" s="2" t="s">
@@ -1598,7 +1570,7 @@
       <c r="I18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J18" s="20" t="s">
+      <c r="J18" s="13" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1615,7 +1587,7 @@
       <c r="D19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="1">
         <v>1</v>
       </c>
       <c r="F19" s="2" t="s">
@@ -1630,7 +1602,7 @@
       <c r="I19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J19" s="20" t="s">
+      <c r="J19" s="13" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1647,7 +1619,7 @@
       <c r="D20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="1">
         <v>1</v>
       </c>
       <c r="F20" s="2" t="s">
@@ -1662,7 +1634,7 @@
       <c r="I20" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="J20" s="20" t="s">
+      <c r="J20" s="13" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1679,7 +1651,7 @@
       <c r="D21" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="1">
         <v>1</v>
       </c>
       <c r="F21" s="2" t="s">
@@ -1694,7 +1666,7 @@
       <c r="I21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J21" s="20" t="s">
+      <c r="J21" s="13" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1711,7 +1683,7 @@
       <c r="D22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E22" s="22">
+      <c r="E22" s="1">
         <v>1</v>
       </c>
       <c r="F22" s="2" t="s">
@@ -1726,7 +1698,7 @@
       <c r="I22" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J22" s="20" t="s">
+      <c r="J22" s="13" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1743,7 +1715,7 @@
       <c r="D23" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E23" s="22">
+      <c r="E23" s="1">
         <v>1</v>
       </c>
       <c r="F23" s="2" t="s">
@@ -1758,44 +1730,77 @@
       <c r="I23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J23" s="20" t="s">
+      <c r="J23" s="13" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="49" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+    <row r="24" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" s="10" t="s">
+      <c r="C24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="14">
         <v>1</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" s="10" t="s">
+      <c r="F24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I24" s="11" t="s">
+      <c r="I24" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J24" s="21" t="s">
+      <c r="J24" s="22" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E25" s="24"/>
+    <row r="25" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="14">
+        <v>1</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J25" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E26" s="15"/>
+      <c r="I26" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>